<commit_message>
chore(sync): PNG 素材資料夾改名（MAT -> MAT, Tinyed）並同步母版與 DB
- data/templates/SLI_ELI letter PNG (MAT) -> (MAT, Tinyed)：5 個製圖 PNG 素材資料夾改名（內容不變）
- data/templates/cainiao-sli-eli-template.xlsx：母版再更新（103 KB -> 95.9 KB）
- data/templates/shipper-role-summary-2026.xlsx：同步最新 report 工作檔
- database.db / db/sessions.db：同步本機資料（pre-commit 自動匯出 db/db-dump.sql）
- FILE_INVENTORY.md：執行 npm run sync 重新產生
</commit_message>
<xml_diff>
--- a/data/templates/cainiao-sli-eli-template.xlsx
+++ b/data/templates/cainiao-sli-eli-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\xls file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\AGL-Web-Portal\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6345F5B-98C9-450D-A5E0-401E16950B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D01E3F-15C4-4885-B9C6-AE5911DABC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30270" yWindow="885" windowWidth="21615" windowHeight="13755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4770" yWindow="1515" windowWidth="21615" windowHeight="13755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="air" sheetId="1" r:id="rId1"/>
@@ -2059,7 +2059,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="238">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2243,6 +2243,213 @@
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="178" fontId="31" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="37" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
@@ -2488,214 +2695,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="178" fontId="31" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="36" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="37" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="51" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5217,56 +5216,241 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1352551</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>37702</xdr:rowOff>
+      <xdr:colOff>1321044</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>48358</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2076451</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Picture 14">
+    <xdr:ext cx="909398" cy="915993"/>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="20" name="群組 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{633A03CE-C0C0-0797-712A-4FEC93AB14DE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A2CF460-AA14-475C-8254-F2CA6B78FE07}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr>
+          <a:grpSpLocks/>
+        </xdr:cNvGrpSpPr>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2019301" y="14048977"/>
-          <a:ext cx="723900" cy="743348"/>
+          <a:off x="1987794" y="13925550"/>
+          <a:ext cx="909398" cy="915993"/>
+          <a:chOff x="6534152" y="1200149"/>
+          <a:chExt cx="3734388" cy="3781066"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="" fLocksText="0">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="21" name="橢圓 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BD5F2A5-B1E1-DABD-21D3-83016C5338EA}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks noChangeAspect="1"/>
+          </xdr:cNvSpPr>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7305562" y="1981201"/>
+            <a:ext cx="2191572" cy="2218966"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="none" lIns="36000" tIns="36000" rIns="36000" bIns="36000" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:endParaRPr lang="en-US" altLang="en-US" sz="2700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="22" name="橢圓 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65CD7C75-F4DA-2858-164E-9CCD3D762EF7}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6534152" y="1200149"/>
+            <a:ext cx="3734388" cy="3781066"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr">
+            <a:prstTxWarp prst="textCircle">
+              <a:avLst/>
+            </a:prstTxWarp>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:fld id="{94C76B59-6E22-4A7D-B5BD-2AE0469CF5A1}" type="TxLink">
+              <a:rPr lang="en-US" altLang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+                <a:ln w="0"/>
+                <a:solidFill>
+                  <a:srgbClr val="002060"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="l"/>
+              <a:t>* KIM LUNG SUPPLY CHAIN (GUANGZHOU) LIMITED.</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" altLang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="標楷體" panose="03000509000000000000" pitchFamily="65" charset="-120"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="23" name="橢圓 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C5F2502-D923-AFDB-1C7F-52E6B28E3846}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6668091" y="1335762"/>
+            <a:ext cx="3466516" cy="3509842"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1100" b="0" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:schemeClr val="dk1">
+                    <a:alpha val="40000"/>
+                  </a:schemeClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5352,7 +5536,7 @@
           <xdr:col>0</xdr:col>
           <xdr:colOff>238125</xdr:colOff>
           <xdr:row>29</xdr:row>
-          <xdr:rowOff>104776</xdr:rowOff>
+          <xdr:rowOff>104775</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5486,7 +5670,7 @@
           <xdr:col>0</xdr:col>
           <xdr:colOff>238125</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>28576</xdr:rowOff>
+          <xdr:rowOff>28575</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5620,7 +5804,7 @@
           <xdr:col>0</xdr:col>
           <xdr:colOff>257175</xdr:colOff>
           <xdr:row>38</xdr:row>
-          <xdr:rowOff>104774</xdr:rowOff>
+          <xdr:rowOff>104775</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5686,8 +5870,8 @@
         <xdr:to>
           <xdr:col>0</xdr:col>
           <xdr:colOff>257175</xdr:colOff>
-          <xdr:row>40</xdr:row>
-          <xdr:rowOff>153865</xdr:rowOff>
+          <xdr:row>41</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5754,7 +5938,7 @@
           <xdr:col>0</xdr:col>
           <xdr:colOff>257175</xdr:colOff>
           <xdr:row>42</xdr:row>
-          <xdr:rowOff>9524</xdr:rowOff>
+          <xdr:rowOff>9525</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5910,56 +6094,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>256442</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>73269</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>189035</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>47290</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9C7C2ED-20FA-4DA6-B5AD-92C3AB9FC15A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3421673" y="8880231"/>
-          <a:ext cx="723900" cy="743348"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>17</xdr:col>
       <xdr:colOff>117232</xdr:colOff>
       <xdr:row>49</xdr:row>
@@ -5985,7 +6119,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -6008,6 +6142,241 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>87923</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="909398" cy="915993"/>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="5" name="群組 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8974D49-F9C3-434D-869F-C0C3C9655C15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr>
+          <a:grpSpLocks/>
+        </xdr:cNvGrpSpPr>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="3253154" y="8689731"/>
+          <a:ext cx="909398" cy="915993"/>
+          <a:chOff x="6534152" y="1200149"/>
+          <a:chExt cx="3734388" cy="3781066"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="" fLocksText="0">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="橢圓 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46FA48B4-D7D9-1418-E84F-E1AE00FD454F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks noChangeAspect="1"/>
+          </xdr:cNvSpPr>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7305562" y="1981201"/>
+            <a:ext cx="2191572" cy="2218966"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="none" lIns="36000" tIns="36000" rIns="36000" bIns="36000" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:endParaRPr lang="en-US" altLang="en-US" sz="2700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="9" name="橢圓 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFCA994E-F07B-9779-CDF0-57A6417795D6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6534152" y="1200149"/>
+            <a:ext cx="3734388" cy="3781066"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr">
+            <a:prstTxWarp prst="textCircle">
+              <a:avLst/>
+            </a:prstTxWarp>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:fld id="{94C76B59-6E22-4A7D-B5BD-2AE0469CF5A1}" type="TxLink">
+              <a:rPr lang="en-US" altLang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+                <a:ln w="0"/>
+                <a:solidFill>
+                  <a:srgbClr val="002060"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="l"/>
+              <a:t>* KIM LUNG SUPPLY CHAIN (GUANGZHOU) LIMITED.</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" altLang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="標楷體" panose="03000509000000000000" pitchFamily="65" charset="-120"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="10" name="橢圓 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09A387DE-3276-724F-B8CD-CC035D81BD51}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6668091" y="1335762"/>
+            <a:ext cx="3466516" cy="3509842"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1100" b="0" cap="none" spc="0">
+              <a:ln w="0"/>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:schemeClr val="dk1">
+                    <a:alpha val="40000"/>
+                  </a:schemeClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -6291,7 +6660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -6318,13 +6687,13 @@
       <c r="I1" s="4"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="198" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="115" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="115" t="s">
+      <c r="C2" s="184" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="7" t="s">
@@ -6333,144 +6702,144 @@
       <c r="E2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="130" t="s">
+      <c r="F2" s="199" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="131"/>
-      <c r="H2" s="134"/>
-      <c r="I2" s="135"/>
+      <c r="G2" s="200"/>
+      <c r="H2" s="203"/>
+      <c r="I2" s="204"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="129"/>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="136" t="s">
+      <c r="A3" s="198"/>
+      <c r="B3" s="184"/>
+      <c r="C3" s="184"/>
+      <c r="D3" s="205" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="137"/>
-      <c r="F3" s="132"/>
-      <c r="G3" s="133"/>
-      <c r="H3" s="133"/>
-      <c r="I3" s="141"/>
+      <c r="E3" s="206"/>
+      <c r="F3" s="201"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="210"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="129"/>
-      <c r="B4" s="115"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="138"/>
-      <c r="E4" s="137"/>
-      <c r="F4" s="132"/>
-      <c r="G4" s="133"/>
-      <c r="H4" s="142"/>
-      <c r="I4" s="143"/>
+      <c r="A4" s="198"/>
+      <c r="B4" s="184"/>
+      <c r="C4" s="184"/>
+      <c r="D4" s="207"/>
+      <c r="E4" s="206"/>
+      <c r="F4" s="201"/>
+      <c r="G4" s="202"/>
+      <c r="H4" s="211"/>
+      <c r="I4" s="212"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="129"/>
-      <c r="B5" s="115"/>
-      <c r="C5" s="115"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="133"/>
-      <c r="H5" s="144"/>
-      <c r="I5" s="145"/>
+      <c r="A5" s="198"/>
+      <c r="B5" s="184"/>
+      <c r="C5" s="184"/>
+      <c r="D5" s="207"/>
+      <c r="E5" s="206"/>
+      <c r="F5" s="201"/>
+      <c r="G5" s="202"/>
+      <c r="H5" s="213"/>
+      <c r="I5" s="214"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="129"/>
-      <c r="B6" s="115"/>
-      <c r="C6" s="115"/>
-      <c r="D6" s="138"/>
-      <c r="E6" s="137"/>
-      <c r="F6" s="146"/>
-      <c r="G6" s="147"/>
-      <c r="H6" s="147"/>
-      <c r="I6" s="148"/>
+      <c r="A6" s="198"/>
+      <c r="B6" s="184"/>
+      <c r="C6" s="184"/>
+      <c r="D6" s="207"/>
+      <c r="E6" s="206"/>
+      <c r="F6" s="215"/>
+      <c r="G6" s="216"/>
+      <c r="H6" s="216"/>
+      <c r="I6" s="217"/>
     </row>
     <row r="7" spans="1:9" ht="29.25" customHeight="1">
-      <c r="A7" s="129"/>
-      <c r="B7" s="115"/>
-      <c r="C7" s="115"/>
-      <c r="D7" s="139"/>
-      <c r="E7" s="140"/>
-      <c r="F7" s="146"/>
-      <c r="G7" s="147"/>
-      <c r="H7" s="147"/>
-      <c r="I7" s="148"/>
+      <c r="A7" s="198"/>
+      <c r="B7" s="184"/>
+      <c r="C7" s="184"/>
+      <c r="D7" s="208"/>
+      <c r="E7" s="209"/>
+      <c r="F7" s="215"/>
+      <c r="G7" s="216"/>
+      <c r="H7" s="216"/>
+      <c r="I7" s="217"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="129"/>
-      <c r="B8" s="115"/>
-      <c r="C8" s="115"/>
+      <c r="A8" s="198"/>
+      <c r="B8" s="184"/>
+      <c r="C8" s="184"/>
       <c r="D8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="9"/>
-      <c r="F8" s="146"/>
-      <c r="G8" s="147"/>
-      <c r="H8" s="147"/>
-      <c r="I8" s="148"/>
+      <c r="F8" s="215"/>
+      <c r="G8" s="216"/>
+      <c r="H8" s="216"/>
+      <c r="I8" s="217"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="129"/>
-      <c r="B9" s="115"/>
-      <c r="C9" s="115"/>
-      <c r="D9" s="152" t="s">
+      <c r="A9" s="198"/>
+      <c r="B9" s="184"/>
+      <c r="C9" s="184"/>
+      <c r="D9" s="221" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="153"/>
-      <c r="F9" s="146"/>
-      <c r="G9" s="147"/>
-      <c r="H9" s="147"/>
-      <c r="I9" s="148"/>
+      <c r="E9" s="222"/>
+      <c r="F9" s="215"/>
+      <c r="G9" s="216"/>
+      <c r="H9" s="216"/>
+      <c r="I9" s="217"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="129"/>
-      <c r="B10" s="115"/>
-      <c r="C10" s="115"/>
-      <c r="D10" s="152"/>
-      <c r="E10" s="153"/>
-      <c r="F10" s="146"/>
-      <c r="G10" s="147"/>
-      <c r="H10" s="147"/>
-      <c r="I10" s="148"/>
+      <c r="A10" s="198"/>
+      <c r="B10" s="184"/>
+      <c r="C10" s="184"/>
+      <c r="D10" s="221"/>
+      <c r="E10" s="222"/>
+      <c r="F10" s="215"/>
+      <c r="G10" s="216"/>
+      <c r="H10" s="216"/>
+      <c r="I10" s="217"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="129"/>
-      <c r="B11" s="115"/>
-      <c r="C11" s="115"/>
-      <c r="D11" s="152"/>
-      <c r="E11" s="153"/>
-      <c r="F11" s="146"/>
-      <c r="G11" s="147"/>
-      <c r="H11" s="147"/>
-      <c r="I11" s="148"/>
+      <c r="A11" s="198"/>
+      <c r="B11" s="184"/>
+      <c r="C11" s="184"/>
+      <c r="D11" s="221"/>
+      <c r="E11" s="222"/>
+      <c r="F11" s="215"/>
+      <c r="G11" s="216"/>
+      <c r="H11" s="216"/>
+      <c r="I11" s="217"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="129"/>
-      <c r="B12" s="115"/>
-      <c r="C12" s="115"/>
-      <c r="D12" s="152"/>
-      <c r="E12" s="153"/>
-      <c r="F12" s="146"/>
-      <c r="G12" s="147"/>
-      <c r="H12" s="147"/>
-      <c r="I12" s="148"/>
+      <c r="A12" s="198"/>
+      <c r="B12" s="184"/>
+      <c r="C12" s="184"/>
+      <c r="D12" s="221"/>
+      <c r="E12" s="222"/>
+      <c r="F12" s="215"/>
+      <c r="G12" s="216"/>
+      <c r="H12" s="216"/>
+      <c r="I12" s="217"/>
     </row>
     <row r="13" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A13" s="129"/>
-      <c r="B13" s="115"/>
-      <c r="C13" s="115"/>
-      <c r="D13" s="154"/>
-      <c r="E13" s="155"/>
-      <c r="F13" s="149"/>
-      <c r="G13" s="150"/>
-      <c r="H13" s="150"/>
-      <c r="I13" s="151"/>
+      <c r="A13" s="198"/>
+      <c r="B13" s="184"/>
+      <c r="C13" s="184"/>
+      <c r="D13" s="223"/>
+      <c r="E13" s="224"/>
+      <c r="F13" s="218"/>
+      <c r="G13" s="219"/>
+      <c r="H13" s="219"/>
+      <c r="I13" s="220"/>
     </row>
     <row r="14" spans="1:9" ht="15.95" customHeight="1">
-      <c r="A14" s="129"/>
-      <c r="B14" s="115"/>
-      <c r="C14" s="115"/>
+      <c r="A14" s="198"/>
+      <c r="B14" s="184"/>
+      <c r="C14" s="184"/>
       <c r="D14" s="10" t="s">
         <v>10</v>
       </c>
@@ -6483,24 +6852,24 @@
       <c r="I14" s="16"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="129"/>
-      <c r="B15" s="115"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="152" t="s">
+      <c r="A15" s="198"/>
+      <c r="B15" s="184"/>
+      <c r="C15" s="184"/>
+      <c r="D15" s="221" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="156"/>
+      <c r="E15" s="225"/>
       <c r="F15" s="17"/>
       <c r="G15" s="18"/>
       <c r="H15" s="18"/>
       <c r="I15" s="19"/>
     </row>
     <row r="16" spans="1:9" ht="15.95" customHeight="1">
-      <c r="A16" s="129"/>
-      <c r="B16" s="115"/>
-      <c r="C16" s="115"/>
-      <c r="D16" s="157"/>
-      <c r="E16" s="156"/>
+      <c r="A16" s="198"/>
+      <c r="B16" s="184"/>
+      <c r="C16" s="184"/>
+      <c r="D16" s="226"/>
+      <c r="E16" s="225"/>
       <c r="F16" s="14" t="s">
         <v>13</v>
       </c>
@@ -6509,158 +6878,158 @@
       <c r="I16" s="21"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="129"/>
-      <c r="B17" s="115"/>
-      <c r="C17" s="115"/>
-      <c r="D17" s="157"/>
-      <c r="E17" s="156"/>
+      <c r="A17" s="198"/>
+      <c r="B17" s="184"/>
+      <c r="C17" s="184"/>
+      <c r="D17" s="226"/>
+      <c r="E17" s="225"/>
       <c r="F17" s="22"/>
       <c r="G17" s="23"/>
       <c r="H17" s="23"/>
       <c r="I17" s="24"/>
     </row>
     <row r="18" spans="1:9" ht="15.95" customHeight="1">
-      <c r="A18" s="129"/>
-      <c r="B18" s="115"/>
-      <c r="C18" s="115"/>
-      <c r="D18" s="157"/>
-      <c r="E18" s="156"/>
+      <c r="A18" s="198"/>
+      <c r="B18" s="184"/>
+      <c r="C18" s="184"/>
+      <c r="D18" s="226"/>
+      <c r="E18" s="225"/>
       <c r="F18" s="14"/>
       <c r="G18" s="20"/>
       <c r="H18" s="20"/>
       <c r="I18" s="21"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="129"/>
-      <c r="B19" s="115"/>
-      <c r="C19" s="115"/>
-      <c r="D19" s="157"/>
-      <c r="E19" s="156"/>
+      <c r="A19" s="198"/>
+      <c r="B19" s="184"/>
+      <c r="C19" s="184"/>
+      <c r="D19" s="226"/>
+      <c r="E19" s="225"/>
       <c r="F19" s="22"/>
       <c r="G19" s="23"/>
       <c r="H19" s="23"/>
       <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="129"/>
-      <c r="B20" s="115"/>
-      <c r="C20" s="115"/>
-      <c r="D20" s="157"/>
-      <c r="E20" s="156"/>
-      <c r="F20" s="158" t="s">
+      <c r="A20" s="198"/>
+      <c r="B20" s="184"/>
+      <c r="C20" s="184"/>
+      <c r="D20" s="226"/>
+      <c r="E20" s="225"/>
+      <c r="F20" s="227" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="160"/>
-      <c r="H20" s="160"/>
-      <c r="I20" s="161"/>
+      <c r="G20" s="229"/>
+      <c r="H20" s="229"/>
+      <c r="I20" s="230"/>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="129"/>
-      <c r="B21" s="115"/>
-      <c r="C21" s="115"/>
-      <c r="D21" s="157"/>
-      <c r="E21" s="156"/>
-      <c r="F21" s="159"/>
-      <c r="G21" s="162"/>
-      <c r="H21" s="162"/>
-      <c r="I21" s="163"/>
+      <c r="A21" s="198"/>
+      <c r="B21" s="184"/>
+      <c r="C21" s="184"/>
+      <c r="D21" s="226"/>
+      <c r="E21" s="225"/>
+      <c r="F21" s="228"/>
+      <c r="G21" s="231"/>
+      <c r="H21" s="231"/>
+      <c r="I21" s="232"/>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="129"/>
-      <c r="B22" s="115"/>
-      <c r="C22" s="115"/>
+      <c r="A22" s="198"/>
+      <c r="B22" s="184"/>
+      <c r="C22" s="184"/>
       <c r="D22" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E22" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="164" t="s">
+      <c r="F22" s="233" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="165"/>
-      <c r="H22" s="165"/>
-      <c r="I22" s="166"/>
+      <c r="G22" s="234"/>
+      <c r="H22" s="234"/>
+      <c r="I22" s="235"/>
     </row>
     <row r="23" spans="1:9" ht="20.25">
-      <c r="A23" s="129"/>
-      <c r="B23" s="115"/>
-      <c r="C23" s="115"/>
+      <c r="A23" s="198"/>
+      <c r="B23" s="184"/>
+      <c r="C23" s="184"/>
       <c r="D23" s="27" t="s">
         <v>18</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="164"/>
-      <c r="G23" s="167"/>
-      <c r="H23" s="167"/>
-      <c r="I23" s="168"/>
+      <c r="F23" s="233"/>
+      <c r="G23" s="236"/>
+      <c r="H23" s="236"/>
+      <c r="I23" s="237"/>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="129"/>
-      <c r="B24" s="115"/>
-      <c r="C24" s="115"/>
+      <c r="A24" s="198"/>
+      <c r="B24" s="184"/>
+      <c r="C24" s="184"/>
       <c r="D24" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E24" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="F24" s="117" t="s">
+      <c r="F24" s="186" t="s">
         <v>22</v>
       </c>
-      <c r="G24" s="118"/>
-      <c r="H24" s="118"/>
-      <c r="I24" s="119"/>
+      <c r="G24" s="187"/>
+      <c r="H24" s="187"/>
+      <c r="I24" s="188"/>
     </row>
     <row r="25" spans="1:9" ht="20.25">
-      <c r="A25" s="129"/>
-      <c r="B25" s="115"/>
-      <c r="C25" s="115"/>
+      <c r="A25" s="198"/>
+      <c r="B25" s="184"/>
+      <c r="C25" s="184"/>
       <c r="D25" s="27" t="s">
         <v>23</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="117"/>
-      <c r="G25" s="118"/>
-      <c r="H25" s="118"/>
-      <c r="I25" s="119"/>
+      <c r="F25" s="186"/>
+      <c r="G25" s="187"/>
+      <c r="H25" s="187"/>
+      <c r="I25" s="188"/>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" s="129"/>
-      <c r="B26" s="115"/>
-      <c r="C26" s="115"/>
+      <c r="A26" s="198"/>
+      <c r="B26" s="184"/>
+      <c r="C26" s="184"/>
       <c r="D26" s="28" t="s">
         <v>25</v>
       </c>
       <c r="E26" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="117"/>
-      <c r="G26" s="118"/>
-      <c r="H26" s="118"/>
-      <c r="I26" s="119"/>
+      <c r="F26" s="186"/>
+      <c r="G26" s="187"/>
+      <c r="H26" s="187"/>
+      <c r="I26" s="188"/>
     </row>
     <row r="27" spans="1:9" ht="20.25">
-      <c r="A27" s="129"/>
-      <c r="B27" s="115"/>
-      <c r="C27" s="115"/>
+      <c r="A27" s="198"/>
+      <c r="B27" s="184"/>
+      <c r="C27" s="184"/>
       <c r="D27" s="27" t="s">
         <v>27</v>
       </c>
       <c r="E27" s="29"/>
-      <c r="F27" s="120"/>
-      <c r="G27" s="121"/>
-      <c r="H27" s="121"/>
-      <c r="I27" s="122"/>
+      <c r="F27" s="189"/>
+      <c r="G27" s="190"/>
+      <c r="H27" s="190"/>
+      <c r="I27" s="191"/>
     </row>
     <row r="28" spans="1:9" ht="24.75" customHeight="1">
-      <c r="A28" s="129"/>
-      <c r="B28" s="115"/>
-      <c r="C28" s="115"/>
+      <c r="A28" s="198"/>
+      <c r="B28" s="184"/>
+      <c r="C28" s="184"/>
       <c r="D28" s="30" t="s">
         <v>28</v>
       </c>
@@ -6670,10 +7039,10 @@
       <c r="F28" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="G28" s="123" t="s">
+      <c r="G28" s="192" t="s">
         <v>31</v>
       </c>
-      <c r="H28" s="123"/>
+      <c r="H28" s="192"/>
       <c r="I28" s="32" t="s">
         <v>32</v>
       </c>
@@ -6683,340 +7052,340 @@
       <c r="B29" s="33"/>
       <c r="C29" s="33"/>
       <c r="D29" s="34"/>
-      <c r="E29" s="124" t="s">
+      <c r="E29" s="193" t="s">
         <v>33</v>
       </c>
       <c r="F29" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="G29" s="127" t="s">
+      <c r="G29" s="196" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="128"/>
+      <c r="H29" s="197"/>
       <c r="I29" s="34"/>
     </row>
     <row r="30" spans="1:9" ht="18">
       <c r="A30" s="33"/>
-      <c r="B30" s="115" t="s">
+      <c r="B30" s="184" t="s">
         <v>36</v>
       </c>
-      <c r="C30" s="116" t="s">
+      <c r="C30" s="185" t="s">
         <v>37</v>
       </c>
       <c r="D30" s="34"/>
-      <c r="E30" s="125"/>
+      <c r="E30" s="194"/>
       <c r="F30" s="36"/>
-      <c r="G30" s="110"/>
-      <c r="H30" s="111"/>
+      <c r="G30" s="179"/>
+      <c r="H30" s="180"/>
       <c r="I30" s="37"/>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="11"/>
-      <c r="B31" s="115"/>
-      <c r="C31" s="116"/>
+      <c r="B31" s="184"/>
+      <c r="C31" s="185"/>
       <c r="D31" s="37"/>
-      <c r="E31" s="125"/>
+      <c r="E31" s="194"/>
       <c r="F31" s="38"/>
-      <c r="G31" s="110"/>
-      <c r="H31" s="111"/>
+      <c r="G31" s="179"/>
+      <c r="H31" s="180"/>
       <c r="I31" s="37"/>
     </row>
     <row r="32" spans="1:9" ht="18">
       <c r="A32" s="11"/>
-      <c r="B32" s="115"/>
-      <c r="C32" s="116"/>
+      <c r="B32" s="184"/>
+      <c r="C32" s="185"/>
       <c r="D32" s="39"/>
-      <c r="E32" s="125"/>
+      <c r="E32" s="194"/>
       <c r="F32" s="38"/>
-      <c r="G32" s="110"/>
-      <c r="H32" s="111"/>
+      <c r="G32" s="179"/>
+      <c r="H32" s="180"/>
       <c r="I32" s="37"/>
     </row>
     <row r="33" spans="1:9" ht="18">
       <c r="A33" s="11"/>
-      <c r="B33" s="115"/>
-      <c r="C33" s="116"/>
+      <c r="B33" s="184"/>
+      <c r="C33" s="185"/>
       <c r="D33" s="39"/>
-      <c r="E33" s="125"/>
+      <c r="E33" s="194"/>
       <c r="F33" s="38"/>
-      <c r="G33" s="110"/>
-      <c r="H33" s="111"/>
+      <c r="G33" s="179"/>
+      <c r="H33" s="180"/>
       <c r="I33" s="37"/>
     </row>
     <row r="34" spans="1:9" ht="18">
       <c r="A34" s="11"/>
-      <c r="B34" s="115"/>
-      <c r="C34" s="116"/>
+      <c r="B34" s="184"/>
+      <c r="C34" s="185"/>
       <c r="D34" s="39"/>
-      <c r="E34" s="125"/>
+      <c r="E34" s="194"/>
       <c r="F34" s="38"/>
-      <c r="G34" s="110"/>
-      <c r="H34" s="111"/>
+      <c r="G34" s="179"/>
+      <c r="H34" s="180"/>
       <c r="I34" s="37"/>
     </row>
     <row r="35" spans="1:9" ht="18">
       <c r="A35" s="11"/>
-      <c r="B35" s="115"/>
-      <c r="C35" s="116"/>
+      <c r="B35" s="184"/>
+      <c r="C35" s="185"/>
       <c r="D35" s="39"/>
-      <c r="E35" s="125"/>
+      <c r="E35" s="194"/>
       <c r="F35" s="38"/>
-      <c r="G35" s="110"/>
-      <c r="H35" s="111"/>
+      <c r="G35" s="179"/>
+      <c r="H35" s="180"/>
       <c r="I35" s="37"/>
     </row>
     <row r="36" spans="1:9" ht="18">
       <c r="A36" s="11"/>
-      <c r="B36" s="115"/>
-      <c r="C36" s="116"/>
+      <c r="B36" s="184"/>
+      <c r="C36" s="185"/>
       <c r="D36" s="39"/>
-      <c r="E36" s="125"/>
+      <c r="E36" s="194"/>
       <c r="F36" s="38"/>
-      <c r="G36" s="110"/>
-      <c r="H36" s="111"/>
+      <c r="G36" s="179"/>
+      <c r="H36" s="180"/>
       <c r="I36" s="37"/>
     </row>
     <row r="37" spans="1:9" ht="18">
       <c r="A37" s="11"/>
-      <c r="B37" s="115"/>
-      <c r="C37" s="116"/>
+      <c r="B37" s="184"/>
+      <c r="C37" s="185"/>
       <c r="D37" s="39"/>
-      <c r="E37" s="125"/>
+      <c r="E37" s="194"/>
       <c r="F37" s="38"/>
-      <c r="G37" s="110"/>
-      <c r="H37" s="111"/>
+      <c r="G37" s="179"/>
+      <c r="H37" s="180"/>
       <c r="I37" s="37"/>
     </row>
     <row r="38" spans="1:9" ht="18">
       <c r="A38" s="11"/>
-      <c r="B38" s="115"/>
-      <c r="C38" s="116"/>
+      <c r="B38" s="184"/>
+      <c r="C38" s="185"/>
       <c r="D38" s="39"/>
-      <c r="E38" s="125"/>
+      <c r="E38" s="194"/>
       <c r="F38" s="38"/>
-      <c r="G38" s="110"/>
-      <c r="H38" s="111"/>
+      <c r="G38" s="179"/>
+      <c r="H38" s="180"/>
       <c r="I38" s="37"/>
     </row>
     <row r="39" spans="1:9" ht="18">
       <c r="A39" s="11"/>
-      <c r="B39" s="115"/>
-      <c r="C39" s="116"/>
+      <c r="B39" s="184"/>
+      <c r="C39" s="185"/>
       <c r="D39" s="39"/>
-      <c r="E39" s="125"/>
+      <c r="E39" s="194"/>
       <c r="F39" s="38"/>
-      <c r="G39" s="110"/>
-      <c r="H39" s="111"/>
+      <c r="G39" s="179"/>
+      <c r="H39" s="180"/>
       <c r="I39" s="37"/>
     </row>
     <row r="40" spans="1:9" ht="18">
-      <c r="A40" s="109" t="s">
+      <c r="A40" s="178" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="115"/>
-      <c r="C40" s="116"/>
+      <c r="B40" s="184"/>
+      <c r="C40" s="185"/>
       <c r="D40" s="39"/>
-      <c r="E40" s="125"/>
+      <c r="E40" s="194"/>
       <c r="F40" s="38"/>
-      <c r="G40" s="110"/>
-      <c r="H40" s="111"/>
+      <c r="G40" s="179"/>
+      <c r="H40" s="180"/>
       <c r="I40" s="37"/>
     </row>
     <row r="41" spans="1:9" ht="18">
-      <c r="A41" s="109"/>
-      <c r="B41" s="115"/>
-      <c r="C41" s="116"/>
+      <c r="A41" s="178"/>
+      <c r="B41" s="184"/>
+      <c r="C41" s="185"/>
       <c r="D41" s="39"/>
-      <c r="E41" s="125"/>
+      <c r="E41" s="194"/>
       <c r="F41" s="38"/>
-      <c r="G41" s="110"/>
-      <c r="H41" s="111"/>
+      <c r="G41" s="179"/>
+      <c r="H41" s="180"/>
       <c r="I41" s="37"/>
     </row>
     <row r="42" spans="1:9" ht="18">
-      <c r="A42" s="109"/>
-      <c r="B42" s="115"/>
-      <c r="C42" s="116"/>
+      <c r="A42" s="178"/>
+      <c r="B42" s="184"/>
+      <c r="C42" s="185"/>
       <c r="D42" s="39"/>
-      <c r="E42" s="125"/>
+      <c r="E42" s="194"/>
       <c r="F42" s="38"/>
-      <c r="G42" s="110"/>
-      <c r="H42" s="111"/>
+      <c r="G42" s="179"/>
+      <c r="H42" s="180"/>
       <c r="I42" s="37"/>
     </row>
     <row r="43" spans="1:9" ht="18">
-      <c r="A43" s="109"/>
-      <c r="B43" s="115"/>
-      <c r="C43" s="116"/>
+      <c r="A43" s="178"/>
+      <c r="B43" s="184"/>
+      <c r="C43" s="185"/>
       <c r="D43" s="39"/>
-      <c r="E43" s="125"/>
+      <c r="E43" s="194"/>
       <c r="F43" s="38"/>
-      <c r="G43" s="110"/>
-      <c r="H43" s="111"/>
+      <c r="G43" s="179"/>
+      <c r="H43" s="180"/>
       <c r="I43" s="37"/>
     </row>
     <row r="44" spans="1:9" ht="18">
-      <c r="A44" s="109"/>
-      <c r="B44" s="115"/>
-      <c r="C44" s="116"/>
+      <c r="A44" s="178"/>
+      <c r="B44" s="184"/>
+      <c r="C44" s="185"/>
       <c r="D44" s="39"/>
-      <c r="E44" s="125"/>
+      <c r="E44" s="194"/>
       <c r="F44" s="38"/>
-      <c r="G44" s="110"/>
-      <c r="H44" s="111"/>
+      <c r="G44" s="179"/>
+      <c r="H44" s="180"/>
       <c r="I44" s="37"/>
     </row>
     <row r="45" spans="1:9" ht="18">
-      <c r="A45" s="109"/>
-      <c r="B45" s="115"/>
-      <c r="C45" s="116"/>
+      <c r="A45" s="178"/>
+      <c r="B45" s="184"/>
+      <c r="C45" s="185"/>
       <c r="D45" s="41"/>
-      <c r="E45" s="126"/>
+      <c r="E45" s="195"/>
       <c r="F45" s="42"/>
-      <c r="G45" s="110"/>
-      <c r="H45" s="111"/>
+      <c r="G45" s="179"/>
+      <c r="H45" s="180"/>
       <c r="I45" s="37"/>
     </row>
     <row r="46" spans="1:9">
-      <c r="A46" s="109"/>
-      <c r="B46" s="115"/>
-      <c r="C46" s="116"/>
-      <c r="D46" s="112" t="s">
+      <c r="A46" s="178"/>
+      <c r="B46" s="184"/>
+      <c r="C46" s="185"/>
+      <c r="D46" s="181" t="s">
         <v>39</v>
       </c>
-      <c r="E46" s="113"/>
-      <c r="F46" s="113"/>
-      <c r="G46" s="113"/>
-      <c r="H46" s="113"/>
-      <c r="I46" s="114"/>
+      <c r="E46" s="182"/>
+      <c r="F46" s="182"/>
+      <c r="G46" s="182"/>
+      <c r="H46" s="182"/>
+      <c r="I46" s="183"/>
     </row>
     <row r="47" spans="1:9">
-      <c r="A47" s="109"/>
-      <c r="B47" s="115"/>
-      <c r="C47" s="116"/>
-      <c r="D47" s="90" t="s">
+      <c r="A47" s="178"/>
+      <c r="B47" s="184"/>
+      <c r="C47" s="185"/>
+      <c r="D47" s="159" t="s">
         <v>40</v>
       </c>
-      <c r="E47" s="91"/>
-      <c r="F47" s="91"/>
-      <c r="G47" s="91"/>
-      <c r="H47" s="91"/>
-      <c r="I47" s="92"/>
+      <c r="E47" s="160"/>
+      <c r="F47" s="160"/>
+      <c r="G47" s="160"/>
+      <c r="H47" s="160"/>
+      <c r="I47" s="161"/>
     </row>
     <row r="48" spans="1:9" ht="15">
-      <c r="A48" s="109"/>
-      <c r="B48" s="115"/>
-      <c r="C48" s="116"/>
-      <c r="D48" s="90" t="s">
+      <c r="A48" s="178"/>
+      <c r="B48" s="184"/>
+      <c r="C48" s="185"/>
+      <c r="D48" s="159" t="s">
         <v>41</v>
       </c>
-      <c r="E48" s="91"/>
-      <c r="F48" s="91"/>
-      <c r="G48" s="91"/>
-      <c r="H48" s="91"/>
-      <c r="I48" s="92"/>
+      <c r="E48" s="160"/>
+      <c r="F48" s="160"/>
+      <c r="G48" s="160"/>
+      <c r="H48" s="160"/>
+      <c r="I48" s="161"/>
     </row>
     <row r="49" spans="1:9" ht="15">
-      <c r="A49" s="109"/>
-      <c r="B49" s="115"/>
-      <c r="C49" s="116"/>
-      <c r="D49" s="90" t="s">
+      <c r="A49" s="178"/>
+      <c r="B49" s="184"/>
+      <c r="C49" s="185"/>
+      <c r="D49" s="159" t="s">
         <v>42</v>
       </c>
-      <c r="E49" s="91"/>
-      <c r="F49" s="91"/>
-      <c r="G49" s="91"/>
-      <c r="H49" s="91"/>
-      <c r="I49" s="92"/>
+      <c r="E49" s="160"/>
+      <c r="F49" s="160"/>
+      <c r="G49" s="160"/>
+      <c r="H49" s="160"/>
+      <c r="I49" s="161"/>
     </row>
     <row r="50" spans="1:9" ht="15">
-      <c r="A50" s="109"/>
-      <c r="B50" s="115"/>
-      <c r="C50" s="116"/>
-      <c r="D50" s="93" t="s">
+      <c r="A50" s="178"/>
+      <c r="B50" s="184"/>
+      <c r="C50" s="185"/>
+      <c r="D50" s="162" t="s">
         <v>43</v>
       </c>
-      <c r="E50" s="94"/>
-      <c r="F50" s="94"/>
-      <c r="G50" s="94"/>
-      <c r="H50" s="94"/>
-      <c r="I50" s="95"/>
+      <c r="E50" s="163"/>
+      <c r="F50" s="163"/>
+      <c r="G50" s="163"/>
+      <c r="H50" s="163"/>
+      <c r="I50" s="164"/>
     </row>
     <row r="51" spans="1:9" ht="15">
-      <c r="A51" s="109"/>
-      <c r="B51" s="115"/>
-      <c r="C51" s="116"/>
-      <c r="D51" s="96" t="s">
+      <c r="A51" s="178"/>
+      <c r="B51" s="184"/>
+      <c r="C51" s="185"/>
+      <c r="D51" s="165" t="s">
         <v>44</v>
       </c>
-      <c r="E51" s="97"/>
-      <c r="F51" s="96" t="s">
+      <c r="E51" s="166"/>
+      <c r="F51" s="165" t="s">
         <v>45</v>
       </c>
-      <c r="G51" s="98"/>
-      <c r="H51" s="98"/>
-      <c r="I51" s="97"/>
+      <c r="G51" s="167"/>
+      <c r="H51" s="167"/>
+      <c r="I51" s="166"/>
     </row>
     <row r="52" spans="1:9" ht="15">
-      <c r="A52" s="109"/>
-      <c r="B52" s="115"/>
-      <c r="C52" s="116"/>
-      <c r="D52" s="99" t="s">
+      <c r="A52" s="178"/>
+      <c r="B52" s="184"/>
+      <c r="C52" s="185"/>
+      <c r="D52" s="168" t="s">
         <v>46</v>
       </c>
-      <c r="E52" s="100"/>
-      <c r="F52" s="101" t="s">
+      <c r="E52" s="169"/>
+      <c r="F52" s="170" t="s">
         <v>47</v>
       </c>
-      <c r="G52" s="102"/>
-      <c r="H52" s="102"/>
-      <c r="I52" s="103"/>
+      <c r="G52" s="171"/>
+      <c r="H52" s="171"/>
+      <c r="I52" s="172"/>
     </row>
     <row r="53" spans="1:9" ht="15">
-      <c r="A53" s="109"/>
-      <c r="B53" s="115"/>
-      <c r="C53" s="116"/>
-      <c r="D53" s="101" t="s">
+      <c r="A53" s="178"/>
+      <c r="B53" s="184"/>
+      <c r="C53" s="185"/>
+      <c r="D53" s="170" t="s">
         <v>48</v>
       </c>
-      <c r="E53" s="103"/>
-      <c r="F53" s="101" t="s">
+      <c r="E53" s="172"/>
+      <c r="F53" s="170" t="s">
         <v>49</v>
       </c>
-      <c r="G53" s="102"/>
-      <c r="H53" s="102"/>
-      <c r="I53" s="103"/>
+      <c r="G53" s="171"/>
+      <c r="H53" s="171"/>
+      <c r="I53" s="172"/>
     </row>
     <row r="54" spans="1:9" ht="15">
-      <c r="A54" s="109"/>
-      <c r="B54" s="115"/>
-      <c r="C54" s="116"/>
-      <c r="D54" s="96" t="s">
+      <c r="A54" s="178"/>
+      <c r="B54" s="184"/>
+      <c r="C54" s="185"/>
+      <c r="D54" s="165" t="s">
         <v>50</v>
       </c>
-      <c r="E54" s="98"/>
-      <c r="F54" s="98"/>
-      <c r="G54" s="98"/>
-      <c r="H54" s="98"/>
-      <c r="I54" s="97"/>
+      <c r="E54" s="167"/>
+      <c r="F54" s="167"/>
+      <c r="G54" s="167"/>
+      <c r="H54" s="167"/>
+      <c r="I54" s="166"/>
     </row>
     <row r="55" spans="1:9" ht="15">
-      <c r="A55" s="109"/>
-      <c r="B55" s="115"/>
-      <c r="C55" s="116"/>
-      <c r="D55" s="104" t="s">
+      <c r="A55" s="178"/>
+      <c r="B55" s="184"/>
+      <c r="C55" s="185"/>
+      <c r="D55" s="173" t="s">
         <v>51</v>
       </c>
-      <c r="E55" s="105"/>
-      <c r="F55" s="105"/>
-      <c r="G55" s="105"/>
-      <c r="H55" s="105"/>
-      <c r="I55" s="106"/>
+      <c r="E55" s="174"/>
+      <c r="F55" s="174"/>
+      <c r="G55" s="174"/>
+      <c r="H55" s="174"/>
+      <c r="I55" s="175"/>
     </row>
     <row r="56" spans="1:9">
-      <c r="A56" s="109"/>
-      <c r="B56" s="115"/>
-      <c r="C56" s="116"/>
+      <c r="A56" s="178"/>
+      <c r="B56" s="184"/>
+      <c r="C56" s="185"/>
       <c r="D56" s="43" t="s">
         <v>52</v>
       </c>
@@ -7035,9 +7404,9 @@
       <c r="I56" s="46"/>
     </row>
     <row r="57" spans="1:9">
-      <c r="A57" s="109"/>
-      <c r="B57" s="115"/>
-      <c r="C57" s="116"/>
+      <c r="A57" s="178"/>
+      <c r="B57" s="184"/>
+      <c r="C57" s="185"/>
       <c r="D57" s="47"/>
       <c r="E57" s="48"/>
       <c r="F57" s="48"/>
@@ -7046,22 +7415,22 @@
       <c r="I57" s="50"/>
     </row>
     <row r="58" spans="1:9">
-      <c r="A58" s="109"/>
-      <c r="B58" s="115"/>
-      <c r="C58" s="116"/>
+      <c r="A58" s="178"/>
+      <c r="B58" s="184"/>
+      <c r="C58" s="185"/>
       <c r="D58" s="10" t="s">
         <v>57</v>
       </c>
       <c r="E58" s="11"/>
-      <c r="F58" s="107"/>
-      <c r="G58" s="107"/>
-      <c r="H58" s="107"/>
-      <c r="I58" s="108"/>
+      <c r="F58" s="176"/>
+      <c r="G58" s="176"/>
+      <c r="H58" s="176"/>
+      <c r="I58" s="177"/>
     </row>
     <row r="59" spans="1:9">
-      <c r="A59" s="109"/>
-      <c r="B59" s="115"/>
-      <c r="C59" s="116"/>
+      <c r="A59" s="178"/>
+      <c r="B59" s="184"/>
+      <c r="C59" s="185"/>
       <c r="D59" s="51"/>
       <c r="E59" s="52"/>
       <c r="F59" s="52"/>
@@ -7070,9 +7439,9 @@
       <c r="I59" s="48"/>
     </row>
     <row r="60" spans="1:9">
-      <c r="A60" s="109"/>
-      <c r="B60" s="115"/>
-      <c r="C60" s="116"/>
+      <c r="A60" s="178"/>
+      <c r="B60" s="184"/>
+      <c r="C60" s="185"/>
       <c r="D60" s="53" t="s">
         <v>58</v>
       </c>
@@ -7175,7 +7544,7 @@
       <c r="B69" s="40"/>
       <c r="C69" s="56"/>
       <c r="D69" s="57"/>
-      <c r="E69" s="235"/>
+      <c r="E69" s="11"/>
       <c r="F69" s="12"/>
       <c r="G69" s="11"/>
       <c r="H69" s="11"/>
@@ -7233,14 +7602,14 @@
       <c r="A74" s="5"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
-      <c r="D74" s="89" t="s">
+      <c r="D74" s="158" t="s">
         <v>60</v>
       </c>
-      <c r="E74" s="89"/>
-      <c r="F74" s="89"/>
-      <c r="G74" s="89"/>
-      <c r="H74" s="89"/>
-      <c r="I74" s="89"/>
+      <c r="E74" s="158"/>
+      <c r="F74" s="158"/>
+      <c r="G74" s="158"/>
+      <c r="H74" s="158"/>
+      <c r="I74" s="158"/>
     </row>
     <row r="75" spans="1:9" ht="15">
       <c r="A75" s="5"/>
@@ -7252,6 +7621,21 @@
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="E78" s="11"/>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="E79" s="11"/>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="E80" s="11"/>
+    </row>
+    <row r="81" spans="5:5">
+      <c r="E81" s="11"/>
+    </row>
+    <row r="82" spans="5:5">
+      <c r="E82" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -7795,98 +8179,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="20.25">
-      <c r="A1" s="236" t="s">
+      <c r="A1" s="152" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="237"/>
-      <c r="C1" s="237"/>
-      <c r="D1" s="237"/>
-      <c r="E1" s="237"/>
-      <c r="F1" s="237"/>
-      <c r="G1" s="237"/>
-      <c r="H1" s="237"/>
-      <c r="I1" s="237"/>
-      <c r="J1" s="237"/>
-      <c r="K1" s="237"/>
-      <c r="L1" s="237"/>
-      <c r="M1" s="237"/>
-      <c r="N1" s="237"/>
-      <c r="O1" s="237"/>
-      <c r="P1" s="237"/>
-      <c r="Q1" s="237"/>
-      <c r="R1" s="237"/>
-      <c r="S1" s="237"/>
-      <c r="T1" s="237"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="153"/>
+      <c r="J1" s="153"/>
+      <c r="K1" s="153"/>
+      <c r="L1" s="153"/>
+      <c r="M1" s="153"/>
+      <c r="N1" s="153"/>
+      <c r="O1" s="153"/>
+      <c r="P1" s="153"/>
+      <c r="Q1" s="153"/>
+      <c r="R1" s="153"/>
+      <c r="S1" s="153"/>
+      <c r="T1" s="153"/>
       <c r="U1" s="62"/>
       <c r="V1" s="62"/>
       <c r="W1" s="62"/>
     </row>
     <row r="2" spans="1:23" hidden="1">
-      <c r="A2" s="232" t="str">
+      <c r="A2" s="154" t="str">
         <f>CONCATENATE("* ",A1)</f>
         <v>* KIM LUNG SUPPLY CHAIN (GUANGZHOU) LIMITED.</v>
       </c>
-      <c r="B2" s="232"/>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="232"/>
-      <c r="H2" s="232"/>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
-      <c r="M2" s="232"/>
-      <c r="N2" s="232"/>
-      <c r="O2" s="232"/>
-      <c r="P2" s="232"/>
-      <c r="Q2" s="232"/>
-      <c r="R2" s="232"/>
-      <c r="S2" s="232"/>
-      <c r="T2" s="232"/>
+      <c r="B2" s="154"/>
+      <c r="C2" s="154"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="154"/>
+      <c r="G2" s="154"/>
+      <c r="H2" s="154"/>
+      <c r="I2" s="154"/>
+      <c r="J2" s="154"/>
+      <c r="K2" s="154"/>
+      <c r="L2" s="154"/>
+      <c r="M2" s="154"/>
+      <c r="N2" s="154"/>
+      <c r="O2" s="154"/>
+      <c r="P2" s="154"/>
+      <c r="Q2" s="154"/>
+      <c r="R2" s="154"/>
+      <c r="S2" s="154"/>
+      <c r="T2" s="154"/>
       <c r="U2" s="63"/>
       <c r="V2" s="63"/>
       <c r="W2" s="63"/>
     </row>
     <row r="3" spans="1:23">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="155" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="238"/>
-      <c r="C3" s="238"/>
-      <c r="D3" s="238"/>
-      <c r="E3" s="238"/>
-      <c r="F3" s="238"/>
-      <c r="G3" s="238"/>
-      <c r="H3" s="238"/>
-      <c r="I3" s="238"/>
-      <c r="J3" s="238"/>
-      <c r="K3" s="238"/>
-      <c r="L3" s="238"/>
-      <c r="M3" s="238"/>
-      <c r="N3" s="238"/>
-      <c r="O3" s="238"/>
-      <c r="P3" s="238"/>
-      <c r="Q3" s="238"/>
-      <c r="R3" s="238"/>
-      <c r="S3" s="238"/>
-      <c r="T3" s="238"/>
+      <c r="B3" s="155"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="155"/>
+      <c r="F3" s="155"/>
+      <c r="G3" s="155"/>
+      <c r="H3" s="155"/>
+      <c r="I3" s="155"/>
+      <c r="J3" s="155"/>
+      <c r="K3" s="155"/>
+      <c r="L3" s="155"/>
+      <c r="M3" s="155"/>
+      <c r="N3" s="155"/>
+      <c r="O3" s="155"/>
+      <c r="P3" s="155"/>
+      <c r="Q3" s="155"/>
+      <c r="R3" s="155"/>
+      <c r="S3" s="155"/>
+      <c r="T3" s="155"/>
       <c r="U3" s="62"/>
       <c r="V3" s="62"/>
       <c r="W3" s="62"/>
     </row>
     <row r="4" spans="1:23" ht="8.1" customHeight="1">
-      <c r="A4" s="233"/>
-      <c r="B4" s="233"/>
-      <c r="C4" s="233"/>
-      <c r="D4" s="233"/>
-      <c r="E4" s="233"/>
-      <c r="F4" s="233"/>
-      <c r="G4" s="233"/>
-      <c r="H4" s="233"/>
-      <c r="I4" s="233"/>
-      <c r="J4" s="233"/>
+      <c r="A4" s="156"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="156"/>
+      <c r="G4" s="156"/>
+      <c r="H4" s="156"/>
+      <c r="I4" s="156"/>
+      <c r="J4" s="156"/>
       <c r="K4" s="65"/>
       <c r="L4" s="65"/>
       <c r="M4" s="65"/>
@@ -7902,57 +8286,57 @@
       <c r="W4" s="65"/>
     </row>
     <row r="5" spans="1:23">
-      <c r="A5" s="234" t="s">
+      <c r="A5" s="157" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="234"/>
-      <c r="C5" s="227" t="s">
+      <c r="B5" s="157"/>
+      <c r="C5" s="147" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="227"/>
-      <c r="E5" s="227"/>
-      <c r="F5" s="227"/>
-      <c r="G5" s="227"/>
-      <c r="H5" s="227"/>
-      <c r="I5" s="227"/>
-      <c r="J5" s="227"/>
-      <c r="K5" s="227"/>
-      <c r="L5" s="227"/>
-      <c r="M5" s="227"/>
-      <c r="N5" s="227"/>
-      <c r="O5" s="227"/>
-      <c r="P5" s="227"/>
-      <c r="Q5" s="227"/>
-      <c r="R5" s="227"/>
-      <c r="S5" s="227"/>
-      <c r="T5" s="227"/>
+      <c r="D5" s="147"/>
+      <c r="E5" s="147"/>
+      <c r="F5" s="147"/>
+      <c r="G5" s="147"/>
+      <c r="H5" s="147"/>
+      <c r="I5" s="147"/>
+      <c r="J5" s="147"/>
+      <c r="K5" s="147"/>
+      <c r="L5" s="147"/>
+      <c r="M5" s="147"/>
+      <c r="N5" s="147"/>
+      <c r="O5" s="147"/>
+      <c r="P5" s="147"/>
+      <c r="Q5" s="147"/>
+      <c r="R5" s="147"/>
+      <c r="S5" s="147"/>
+      <c r="T5" s="147"/>
       <c r="U5" s="62"/>
       <c r="V5" s="62"/>
       <c r="W5" s="62"/>
     </row>
     <row r="6" spans="1:23">
-      <c r="A6" s="226"/>
-      <c r="B6" s="226"/>
-      <c r="C6" s="227" t="s">
+      <c r="A6" s="146"/>
+      <c r="B6" s="146"/>
+      <c r="C6" s="147" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="227"/>
-      <c r="E6" s="227"/>
-      <c r="F6" s="227"/>
-      <c r="G6" s="227"/>
-      <c r="H6" s="227"/>
-      <c r="I6" s="227"/>
-      <c r="J6" s="227"/>
-      <c r="K6" s="227"/>
-      <c r="L6" s="227"/>
-      <c r="M6" s="227"/>
-      <c r="N6" s="227"/>
-      <c r="O6" s="227"/>
-      <c r="P6" s="227"/>
-      <c r="Q6" s="227"/>
-      <c r="R6" s="227"/>
-      <c r="S6" s="227"/>
-      <c r="T6" s="227"/>
+      <c r="D6" s="147"/>
+      <c r="E6" s="147"/>
+      <c r="F6" s="147"/>
+      <c r="G6" s="147"/>
+      <c r="H6" s="147"/>
+      <c r="I6" s="147"/>
+      <c r="J6" s="147"/>
+      <c r="K6" s="147"/>
+      <c r="L6" s="147"/>
+      <c r="M6" s="147"/>
+      <c r="N6" s="147"/>
+      <c r="O6" s="147"/>
+      <c r="P6" s="147"/>
+      <c r="Q6" s="147"/>
+      <c r="R6" s="147"/>
+      <c r="S6" s="147"/>
+      <c r="T6" s="147"/>
       <c r="U6" s="62"/>
       <c r="V6" s="62"/>
       <c r="W6" s="62"/>
@@ -7985,46 +8369,46 @@
       <c r="W7" s="67"/>
     </row>
     <row r="8" spans="1:23">
-      <c r="A8" s="207" t="s">
+      <c r="A8" s="127" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="207"/>
-      <c r="C8" s="207"/>
-      <c r="D8" s="207"/>
-      <c r="E8" s="207"/>
-      <c r="F8" s="228" t="s">
+      <c r="B8" s="127"/>
+      <c r="C8" s="127"/>
+      <c r="D8" s="127"/>
+      <c r="E8" s="127"/>
+      <c r="F8" s="148" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="228"/>
-      <c r="H8" s="228"/>
-      <c r="I8" s="228"/>
-      <c r="J8" s="228"/>
-      <c r="K8" s="207" t="s">
+      <c r="G8" s="148"/>
+      <c r="H8" s="148"/>
+      <c r="I8" s="148"/>
+      <c r="J8" s="148"/>
+      <c r="K8" s="127" t="s">
         <v>69</v>
       </c>
-      <c r="L8" s="207"/>
-      <c r="M8" s="207"/>
-      <c r="N8" s="207"/>
-      <c r="O8" s="207"/>
-      <c r="P8" s="229" t="s">
+      <c r="L8" s="127"/>
+      <c r="M8" s="127"/>
+      <c r="N8" s="127"/>
+      <c r="O8" s="127"/>
+      <c r="P8" s="149" t="s">
         <v>70</v>
       </c>
-      <c r="Q8" s="229"/>
-      <c r="R8" s="229"/>
-      <c r="S8" s="229"/>
-      <c r="T8" s="229"/>
+      <c r="Q8" s="149"/>
+      <c r="R8" s="149"/>
+      <c r="S8" s="149"/>
+      <c r="T8" s="149"/>
       <c r="U8" s="65"/>
       <c r="V8" s="65"/>
       <c r="W8" s="65"/>
     </row>
     <row r="9" spans="1:23">
-      <c r="A9" s="225" t="s">
+      <c r="A9" s="145" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="230"/>
-      <c r="C9" s="230"/>
-      <c r="D9" s="230"/>
-      <c r="E9" s="230"/>
+      <c r="B9" s="150"/>
+      <c r="C9" s="150"/>
+      <c r="D9" s="150"/>
+      <c r="E9" s="150"/>
       <c r="F9" s="65"/>
       <c r="G9" s="65"/>
       <c r="H9" s="65"/>
@@ -8070,44 +8454,44 @@
       <c r="W10" s="65"/>
     </row>
     <row r="11" spans="1:23">
-      <c r="A11" s="207" t="s">
+      <c r="A11" s="127" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="207"/>
-      <c r="C11" s="207"/>
-      <c r="D11" s="207"/>
-      <c r="E11" s="207"/>
-      <c r="F11" s="231"/>
-      <c r="G11" s="229"/>
-      <c r="H11" s="229"/>
-      <c r="I11" s="229"/>
-      <c r="J11" s="229"/>
-      <c r="K11" s="207" t="s">
+      <c r="B11" s="127"/>
+      <c r="C11" s="127"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="127"/>
+      <c r="F11" s="151"/>
+      <c r="G11" s="149"/>
+      <c r="H11" s="149"/>
+      <c r="I11" s="149"/>
+      <c r="J11" s="149"/>
+      <c r="K11" s="127" t="s">
         <v>73</v>
       </c>
-      <c r="L11" s="207"/>
-      <c r="M11" s="207"/>
-      <c r="N11" s="207"/>
-      <c r="O11" s="207"/>
-      <c r="P11" s="229" t="s">
+      <c r="L11" s="127"/>
+      <c r="M11" s="127"/>
+      <c r="N11" s="127"/>
+      <c r="O11" s="127"/>
+      <c r="P11" s="149" t="s">
         <v>74</v>
       </c>
-      <c r="Q11" s="229"/>
-      <c r="R11" s="229"/>
-      <c r="S11" s="229"/>
-      <c r="T11" s="229"/>
+      <c r="Q11" s="149"/>
+      <c r="R11" s="149"/>
+      <c r="S11" s="149"/>
+      <c r="T11" s="149"/>
       <c r="U11" s="65"/>
       <c r="V11" s="65"/>
       <c r="W11" s="65"/>
     </row>
     <row r="12" spans="1:23">
-      <c r="A12" s="225" t="s">
+      <c r="A12" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="B12" s="225"/>
-      <c r="C12" s="225"/>
-      <c r="D12" s="225"/>
-      <c r="E12" s="225"/>
+      <c r="B12" s="145"/>
+      <c r="C12" s="145"/>
+      <c r="D12" s="145"/>
+      <c r="E12" s="145"/>
       <c r="F12" s="65"/>
       <c r="G12" s="65"/>
       <c r="H12" s="65"/>
@@ -8207,63 +8591,63 @@
       <c r="W15" s="65"/>
     </row>
     <row r="16" spans="1:23">
-      <c r="A16" s="206" t="s">
+      <c r="A16" s="126" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="207"/>
-      <c r="C16" s="217" t="s">
+      <c r="B16" s="127"/>
+      <c r="C16" s="137" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="217"/>
-      <c r="E16" s="217"/>
-      <c r="F16" s="217"/>
-      <c r="G16" s="217"/>
-      <c r="H16" s="217"/>
-      <c r="I16" s="217"/>
-      <c r="J16" s="218"/>
-      <c r="K16" s="206" t="s">
+      <c r="D16" s="137"/>
+      <c r="E16" s="137"/>
+      <c r="F16" s="137"/>
+      <c r="G16" s="137"/>
+      <c r="H16" s="137"/>
+      <c r="I16" s="137"/>
+      <c r="J16" s="138"/>
+      <c r="K16" s="126" t="s">
         <v>78</v>
       </c>
-      <c r="L16" s="207"/>
-      <c r="M16" s="221" t="s">
+      <c r="L16" s="127"/>
+      <c r="M16" s="141" t="s">
         <v>80</v>
       </c>
-      <c r="N16" s="221"/>
-      <c r="O16" s="221"/>
-      <c r="P16" s="221"/>
-      <c r="Q16" s="221"/>
-      <c r="R16" s="221"/>
-      <c r="S16" s="221"/>
-      <c r="T16" s="222"/>
+      <c r="N16" s="141"/>
+      <c r="O16" s="141"/>
+      <c r="P16" s="141"/>
+      <c r="Q16" s="141"/>
+      <c r="R16" s="141"/>
+      <c r="S16" s="141"/>
+      <c r="T16" s="142"/>
       <c r="U16" s="62"/>
       <c r="V16" s="62"/>
       <c r="W16" s="62"/>
     </row>
     <row r="17" spans="1:23">
-      <c r="A17" s="206" t="s">
+      <c r="A17" s="126" t="s">
         <v>81</v>
       </c>
-      <c r="B17" s="207"/>
-      <c r="C17" s="217"/>
-      <c r="D17" s="217"/>
-      <c r="E17" s="217"/>
-      <c r="F17" s="217"/>
-      <c r="G17" s="217"/>
-      <c r="H17" s="217"/>
-      <c r="I17" s="217"/>
-      <c r="J17" s="218"/>
-      <c r="K17" s="206" t="s">
+      <c r="B17" s="127"/>
+      <c r="C17" s="137"/>
+      <c r="D17" s="137"/>
+      <c r="E17" s="137"/>
+      <c r="F17" s="137"/>
+      <c r="G17" s="137"/>
+      <c r="H17" s="137"/>
+      <c r="I17" s="137"/>
+      <c r="J17" s="138"/>
+      <c r="K17" s="126" t="s">
         <v>81</v>
       </c>
-      <c r="L17" s="207"/>
-      <c r="M17" s="221"/>
-      <c r="N17" s="221"/>
-      <c r="O17" s="221"/>
-      <c r="P17" s="221"/>
-      <c r="Q17" s="221"/>
-      <c r="R17" s="221"/>
-      <c r="S17" s="221"/>
-      <c r="T17" s="222"/>
+      <c r="L17" s="127"/>
+      <c r="M17" s="141"/>
+      <c r="N17" s="141"/>
+      <c r="O17" s="141"/>
+      <c r="P17" s="141"/>
+      <c r="Q17" s="141"/>
+      <c r="R17" s="141"/>
+      <c r="S17" s="141"/>
+      <c r="T17" s="142"/>
       <c r="U17" s="62"/>
       <c r="V17" s="62"/>
       <c r="W17" s="62"/>
@@ -8271,24 +8655,24 @@
     <row r="18" spans="1:23">
       <c r="A18" s="73"/>
       <c r="B18" s="62"/>
-      <c r="C18" s="217"/>
-      <c r="D18" s="217"/>
-      <c r="E18" s="217"/>
-      <c r="F18" s="217"/>
-      <c r="G18" s="217"/>
-      <c r="H18" s="217"/>
-      <c r="I18" s="217"/>
-      <c r="J18" s="218"/>
+      <c r="C18" s="137"/>
+      <c r="D18" s="137"/>
+      <c r="E18" s="137"/>
+      <c r="F18" s="137"/>
+      <c r="G18" s="137"/>
+      <c r="H18" s="137"/>
+      <c r="I18" s="137"/>
+      <c r="J18" s="138"/>
       <c r="K18" s="73"/>
       <c r="L18" s="62"/>
-      <c r="M18" s="221"/>
-      <c r="N18" s="221"/>
-      <c r="O18" s="221"/>
-      <c r="P18" s="221"/>
-      <c r="Q18" s="221"/>
-      <c r="R18" s="221"/>
-      <c r="S18" s="221"/>
-      <c r="T18" s="222"/>
+      <c r="M18" s="141"/>
+      <c r="N18" s="141"/>
+      <c r="O18" s="141"/>
+      <c r="P18" s="141"/>
+      <c r="Q18" s="141"/>
+      <c r="R18" s="141"/>
+      <c r="S18" s="141"/>
+      <c r="T18" s="142"/>
       <c r="U18" s="62"/>
       <c r="V18" s="62"/>
       <c r="W18" s="62"/>
@@ -8296,24 +8680,24 @@
     <row r="19" spans="1:23">
       <c r="A19" s="73"/>
       <c r="B19" s="62"/>
-      <c r="C19" s="217"/>
-      <c r="D19" s="217"/>
-      <c r="E19" s="217"/>
-      <c r="F19" s="217"/>
-      <c r="G19" s="217"/>
-      <c r="H19" s="217"/>
-      <c r="I19" s="217"/>
-      <c r="J19" s="218"/>
+      <c r="C19" s="137"/>
+      <c r="D19" s="137"/>
+      <c r="E19" s="137"/>
+      <c r="F19" s="137"/>
+      <c r="G19" s="137"/>
+      <c r="H19" s="137"/>
+      <c r="I19" s="137"/>
+      <c r="J19" s="138"/>
       <c r="K19" s="73"/>
       <c r="L19" s="62"/>
-      <c r="M19" s="221"/>
-      <c r="N19" s="221"/>
-      <c r="O19" s="221"/>
-      <c r="P19" s="221"/>
-      <c r="Q19" s="221"/>
-      <c r="R19" s="221"/>
-      <c r="S19" s="221"/>
-      <c r="T19" s="222"/>
+      <c r="M19" s="141"/>
+      <c r="N19" s="141"/>
+      <c r="O19" s="141"/>
+      <c r="P19" s="141"/>
+      <c r="Q19" s="141"/>
+      <c r="R19" s="141"/>
+      <c r="S19" s="141"/>
+      <c r="T19" s="142"/>
       <c r="U19" s="62"/>
       <c r="V19" s="62"/>
       <c r="W19" s="62"/>
@@ -8321,57 +8705,57 @@
     <row r="20" spans="1:23">
       <c r="A20" s="73"/>
       <c r="B20" s="62"/>
-      <c r="C20" s="219"/>
-      <c r="D20" s="219"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="219"/>
-      <c r="G20" s="219"/>
-      <c r="H20" s="219"/>
-      <c r="I20" s="219"/>
-      <c r="J20" s="220"/>
+      <c r="C20" s="139"/>
+      <c r="D20" s="139"/>
+      <c r="E20" s="139"/>
+      <c r="F20" s="139"/>
+      <c r="G20" s="139"/>
+      <c r="H20" s="139"/>
+      <c r="I20" s="139"/>
+      <c r="J20" s="140"/>
       <c r="K20" s="73"/>
       <c r="L20" s="62"/>
-      <c r="M20" s="223"/>
-      <c r="N20" s="223"/>
-      <c r="O20" s="223"/>
-      <c r="P20" s="223"/>
-      <c r="Q20" s="223"/>
-      <c r="R20" s="223"/>
-      <c r="S20" s="223"/>
-      <c r="T20" s="224"/>
+      <c r="M20" s="143"/>
+      <c r="N20" s="143"/>
+      <c r="O20" s="143"/>
+      <c r="P20" s="143"/>
+      <c r="Q20" s="143"/>
+      <c r="R20" s="143"/>
+      <c r="S20" s="143"/>
+      <c r="T20" s="144"/>
       <c r="U20" s="62"/>
       <c r="V20" s="62"/>
       <c r="W20" s="62"/>
     </row>
     <row r="21" spans="1:23">
-      <c r="A21" s="206" t="s">
+      <c r="A21" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="207"/>
-      <c r="C21" s="207"/>
-      <c r="D21" s="208" t="s">
+      <c r="B21" s="127"/>
+      <c r="C21" s="127"/>
+      <c r="D21" s="128" t="s">
         <v>83</v>
       </c>
-      <c r="E21" s="209"/>
-      <c r="F21" s="209"/>
-      <c r="G21" s="209"/>
-      <c r="H21" s="209"/>
-      <c r="I21" s="209"/>
-      <c r="J21" s="210"/>
-      <c r="K21" s="206" t="s">
+      <c r="E21" s="129"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="129"/>
+      <c r="H21" s="129"/>
+      <c r="I21" s="129"/>
+      <c r="J21" s="130"/>
+      <c r="K21" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="L21" s="207"/>
-      <c r="M21" s="207"/>
-      <c r="N21" s="211" t="s">
+      <c r="L21" s="127"/>
+      <c r="M21" s="127"/>
+      <c r="N21" s="131" t="s">
         <v>84</v>
       </c>
-      <c r="O21" s="209"/>
-      <c r="P21" s="209"/>
-      <c r="Q21" s="209"/>
-      <c r="R21" s="209"/>
-      <c r="S21" s="209"/>
-      <c r="T21" s="210"/>
+      <c r="O21" s="129"/>
+      <c r="P21" s="129"/>
+      <c r="Q21" s="129"/>
+      <c r="R21" s="129"/>
+      <c r="S21" s="129"/>
+      <c r="T21" s="130"/>
       <c r="U21" s="62"/>
       <c r="V21" s="62"/>
       <c r="W21" s="62"/>
@@ -8455,60 +8839,60 @@
     </row>
     <row r="25" spans="1:23">
       <c r="A25" s="77"/>
-      <c r="B25" s="212" t="s">
+      <c r="B25" s="132" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="213"/>
-      <c r="D25" s="213"/>
-      <c r="E25" s="213"/>
-      <c r="F25" s="213"/>
-      <c r="G25" s="213"/>
-      <c r="H25" s="213"/>
-      <c r="I25" s="213"/>
-      <c r="J25" s="213"/>
+      <c r="C25" s="133"/>
+      <c r="D25" s="133"/>
+      <c r="E25" s="133"/>
+      <c r="F25" s="133"/>
+      <c r="G25" s="133"/>
+      <c r="H25" s="133"/>
+      <c r="I25" s="133"/>
+      <c r="J25" s="133"/>
       <c r="K25" s="78"/>
-      <c r="L25" s="214" t="s">
+      <c r="L25" s="134" t="s">
         <v>87</v>
       </c>
-      <c r="M25" s="215"/>
-      <c r="N25" s="216"/>
-      <c r="O25" s="214" t="s">
+      <c r="M25" s="135"/>
+      <c r="N25" s="136"/>
+      <c r="O25" s="134" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="215"/>
-      <c r="Q25" s="215"/>
-      <c r="R25" s="215"/>
-      <c r="S25" s="215"/>
-      <c r="T25" s="216"/>
+      <c r="P25" s="135"/>
+      <c r="Q25" s="135"/>
+      <c r="R25" s="135"/>
+      <c r="S25" s="135"/>
+      <c r="T25" s="136"/>
       <c r="U25" s="77"/>
       <c r="V25" s="77"/>
       <c r="W25" s="77"/>
     </row>
     <row r="26" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A26" s="79"/>
-      <c r="B26" s="177" t="s">
+      <c r="B26" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="204"/>
-      <c r="D26" s="204"/>
-      <c r="E26" s="204"/>
-      <c r="F26" s="205"/>
-      <c r="G26" s="194" t="s">
+      <c r="C26" s="124"/>
+      <c r="D26" s="124"/>
+      <c r="E26" s="124"/>
+      <c r="F26" s="125"/>
+      <c r="G26" s="114" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="195"/>
-      <c r="I26" s="195"/>
-      <c r="J26" s="195"/>
-      <c r="K26" s="195"/>
-      <c r="L26" s="180"/>
-      <c r="M26" s="181"/>
-      <c r="N26" s="182"/>
-      <c r="O26" s="186"/>
-      <c r="P26" s="187"/>
-      <c r="Q26" s="187"/>
-      <c r="R26" s="187"/>
-      <c r="S26" s="187"/>
-      <c r="T26" s="188"/>
+      <c r="H26" s="115"/>
+      <c r="I26" s="115"/>
+      <c r="J26" s="115"/>
+      <c r="K26" s="115"/>
+      <c r="L26" s="100"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="102"/>
+      <c r="O26" s="106"/>
+      <c r="P26" s="107"/>
+      <c r="Q26" s="107"/>
+      <c r="R26" s="107"/>
+      <c r="S26" s="107"/>
+      <c r="T26" s="108"/>
       <c r="U26" s="79"/>
       <c r="V26" s="79" t="s">
         <v>91</v>
@@ -8517,29 +8901,29 @@
     </row>
     <row r="27" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A27" s="79"/>
-      <c r="B27" s="202" t="s">
+      <c r="B27" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="C27" s="173"/>
-      <c r="D27" s="173"/>
-      <c r="E27" s="173"/>
-      <c r="F27" s="203"/>
-      <c r="G27" s="194" t="s">
+      <c r="C27" s="93"/>
+      <c r="D27" s="93"/>
+      <c r="E27" s="93"/>
+      <c r="F27" s="123"/>
+      <c r="G27" s="114" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="195"/>
-      <c r="I27" s="195"/>
-      <c r="J27" s="195"/>
-      <c r="K27" s="195"/>
-      <c r="L27" s="196"/>
-      <c r="M27" s="197"/>
-      <c r="N27" s="198"/>
-      <c r="O27" s="199"/>
-      <c r="P27" s="200"/>
-      <c r="Q27" s="200"/>
-      <c r="R27" s="200"/>
-      <c r="S27" s="200"/>
-      <c r="T27" s="201"/>
+      <c r="H27" s="115"/>
+      <c r="I27" s="115"/>
+      <c r="J27" s="115"/>
+      <c r="K27" s="115"/>
+      <c r="L27" s="116"/>
+      <c r="M27" s="117"/>
+      <c r="N27" s="118"/>
+      <c r="O27" s="119"/>
+      <c r="P27" s="120"/>
+      <c r="Q27" s="120"/>
+      <c r="R27" s="120"/>
+      <c r="S27" s="120"/>
+      <c r="T27" s="121"/>
       <c r="U27" s="79"/>
       <c r="V27" s="79" t="s">
         <v>94</v>
@@ -8548,29 +8932,29 @@
     </row>
     <row r="28" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A28" s="79"/>
-      <c r="B28" s="192" t="s">
+      <c r="B28" s="112" t="s">
         <v>95</v>
       </c>
-      <c r="C28" s="175"/>
-      <c r="D28" s="175"/>
-      <c r="E28" s="175"/>
-      <c r="F28" s="193"/>
-      <c r="G28" s="194" t="s">
+      <c r="C28" s="95"/>
+      <c r="D28" s="95"/>
+      <c r="E28" s="95"/>
+      <c r="F28" s="113"/>
+      <c r="G28" s="114" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="195"/>
-      <c r="I28" s="195"/>
-      <c r="J28" s="195"/>
-      <c r="K28" s="195"/>
-      <c r="L28" s="183"/>
-      <c r="M28" s="184"/>
-      <c r="N28" s="185"/>
-      <c r="O28" s="189"/>
-      <c r="P28" s="190"/>
-      <c r="Q28" s="190"/>
-      <c r="R28" s="190"/>
-      <c r="S28" s="190"/>
-      <c r="T28" s="191"/>
+      <c r="H28" s="115"/>
+      <c r="I28" s="115"/>
+      <c r="J28" s="115"/>
+      <c r="K28" s="115"/>
+      <c r="L28" s="103"/>
+      <c r="M28" s="104"/>
+      <c r="N28" s="105"/>
+      <c r="O28" s="109"/>
+      <c r="P28" s="110"/>
+      <c r="Q28" s="110"/>
+      <c r="R28" s="110"/>
+      <c r="S28" s="110"/>
+      <c r="T28" s="111"/>
       <c r="U28" s="79"/>
       <c r="V28" s="79" t="s">
         <v>97</v>
@@ -8579,54 +8963,54 @@
     </row>
     <row r="29" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A29" s="79"/>
-      <c r="B29" s="177" t="s">
+      <c r="B29" s="97" t="s">
         <v>98</v>
       </c>
-      <c r="C29" s="178"/>
-      <c r="D29" s="178"/>
-      <c r="E29" s="178"/>
-      <c r="F29" s="178"/>
-      <c r="G29" s="178"/>
-      <c r="H29" s="178"/>
-      <c r="I29" s="178"/>
-      <c r="J29" s="178"/>
-      <c r="K29" s="179"/>
-      <c r="L29" s="180"/>
-      <c r="M29" s="181"/>
-      <c r="N29" s="182"/>
-      <c r="O29" s="186"/>
-      <c r="P29" s="187"/>
-      <c r="Q29" s="187"/>
-      <c r="R29" s="187"/>
-      <c r="S29" s="187"/>
-      <c r="T29" s="188"/>
+      <c r="C29" s="98"/>
+      <c r="D29" s="98"/>
+      <c r="E29" s="98"/>
+      <c r="F29" s="98"/>
+      <c r="G29" s="98"/>
+      <c r="H29" s="98"/>
+      <c r="I29" s="98"/>
+      <c r="J29" s="98"/>
+      <c r="K29" s="99"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="102"/>
+      <c r="O29" s="106"/>
+      <c r="P29" s="107"/>
+      <c r="Q29" s="107"/>
+      <c r="R29" s="107"/>
+      <c r="S29" s="107"/>
+      <c r="T29" s="108"/>
       <c r="U29" s="79"/>
       <c r="V29" s="79"/>
       <c r="W29" s="79"/>
     </row>
     <row r="30" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A30" s="79"/>
-      <c r="B30" s="192" t="s">
+      <c r="B30" s="112" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="175"/>
-      <c r="D30" s="175"/>
-      <c r="E30" s="175"/>
-      <c r="F30" s="175"/>
-      <c r="G30" s="175"/>
-      <c r="H30" s="175"/>
-      <c r="I30" s="175"/>
-      <c r="J30" s="175"/>
-      <c r="K30" s="193"/>
-      <c r="L30" s="183"/>
-      <c r="M30" s="184"/>
-      <c r="N30" s="185"/>
-      <c r="O30" s="189"/>
-      <c r="P30" s="190"/>
-      <c r="Q30" s="190"/>
-      <c r="R30" s="190"/>
-      <c r="S30" s="190"/>
-      <c r="T30" s="191"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="95"/>
+      <c r="E30" s="95"/>
+      <c r="F30" s="95"/>
+      <c r="G30" s="95"/>
+      <c r="H30" s="95"/>
+      <c r="I30" s="95"/>
+      <c r="J30" s="95"/>
+      <c r="K30" s="113"/>
+      <c r="L30" s="103"/>
+      <c r="M30" s="104"/>
+      <c r="N30" s="105"/>
+      <c r="O30" s="109"/>
+      <c r="P30" s="110"/>
+      <c r="Q30" s="110"/>
+      <c r="R30" s="110"/>
+      <c r="S30" s="110"/>
+      <c r="T30" s="111"/>
       <c r="U30" s="82"/>
       <c r="V30" s="82" t="s">
         <v>127</v>
@@ -8635,85 +9019,85 @@
     </row>
     <row r="31" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A31" s="79"/>
-      <c r="B31" s="177" t="s">
+      <c r="B31" s="97" t="s">
         <v>100</v>
       </c>
-      <c r="C31" s="178"/>
-      <c r="D31" s="178"/>
-      <c r="E31" s="178"/>
-      <c r="F31" s="178"/>
-      <c r="G31" s="178"/>
-      <c r="H31" s="178"/>
-      <c r="I31" s="178"/>
-      <c r="J31" s="178"/>
-      <c r="K31" s="179"/>
-      <c r="L31" s="180"/>
-      <c r="M31" s="181"/>
-      <c r="N31" s="182"/>
-      <c r="O31" s="186" t="s">
+      <c r="C31" s="98"/>
+      <c r="D31" s="98"/>
+      <c r="E31" s="98"/>
+      <c r="F31" s="98"/>
+      <c r="G31" s="98"/>
+      <c r="H31" s="98"/>
+      <c r="I31" s="98"/>
+      <c r="J31" s="98"/>
+      <c r="K31" s="99"/>
+      <c r="L31" s="100"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="102"/>
+      <c r="O31" s="106" t="s">
         <v>101</v>
       </c>
-      <c r="P31" s="187"/>
-      <c r="Q31" s="187"/>
-      <c r="R31" s="187"/>
-      <c r="S31" s="187"/>
-      <c r="T31" s="188"/>
+      <c r="P31" s="107"/>
+      <c r="Q31" s="107"/>
+      <c r="R31" s="107"/>
+      <c r="S31" s="107"/>
+      <c r="T31" s="108"/>
       <c r="U31" s="79"/>
       <c r="V31" s="79"/>
       <c r="W31" s="79"/>
     </row>
     <row r="32" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A32" s="79"/>
-      <c r="B32" s="192" t="s">
+      <c r="B32" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="C32" s="175"/>
-      <c r="D32" s="175"/>
-      <c r="E32" s="175"/>
-      <c r="F32" s="175"/>
-      <c r="G32" s="175"/>
-      <c r="H32" s="175"/>
-      <c r="I32" s="175"/>
-      <c r="J32" s="175"/>
-      <c r="K32" s="193"/>
-      <c r="L32" s="183"/>
-      <c r="M32" s="184"/>
-      <c r="N32" s="185"/>
-      <c r="O32" s="189"/>
-      <c r="P32" s="190"/>
-      <c r="Q32" s="190"/>
-      <c r="R32" s="190"/>
-      <c r="S32" s="190"/>
-      <c r="T32" s="191"/>
+      <c r="C32" s="95"/>
+      <c r="D32" s="95"/>
+      <c r="E32" s="95"/>
+      <c r="F32" s="95"/>
+      <c r="G32" s="95"/>
+      <c r="H32" s="95"/>
+      <c r="I32" s="95"/>
+      <c r="J32" s="95"/>
+      <c r="K32" s="113"/>
+      <c r="L32" s="103"/>
+      <c r="M32" s="104"/>
+      <c r="N32" s="105"/>
+      <c r="O32" s="109"/>
+      <c r="P32" s="110"/>
+      <c r="Q32" s="110"/>
+      <c r="R32" s="110"/>
+      <c r="S32" s="110"/>
+      <c r="T32" s="111"/>
       <c r="U32" s="79"/>
       <c r="V32" s="79"/>
       <c r="W32" s="79"/>
     </row>
     <row r="33" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A33" s="79"/>
-      <c r="B33" s="177" t="s">
+      <c r="B33" s="97" t="s">
         <v>103</v>
       </c>
-      <c r="C33" s="178"/>
-      <c r="D33" s="178"/>
-      <c r="E33" s="178"/>
-      <c r="F33" s="179"/>
-      <c r="G33" s="194" t="s">
+      <c r="C33" s="98"/>
+      <c r="D33" s="98"/>
+      <c r="E33" s="98"/>
+      <c r="F33" s="99"/>
+      <c r="G33" s="114" t="s">
         <v>104</v>
       </c>
-      <c r="H33" s="195"/>
-      <c r="I33" s="195"/>
-      <c r="J33" s="195"/>
-      <c r="K33" s="195"/>
-      <c r="L33" s="180"/>
-      <c r="M33" s="181"/>
-      <c r="N33" s="182"/>
-      <c r="O33" s="186"/>
-      <c r="P33" s="187"/>
-      <c r="Q33" s="187"/>
-      <c r="R33" s="187"/>
-      <c r="S33" s="187"/>
-      <c r="T33" s="188"/>
+      <c r="H33" s="115"/>
+      <c r="I33" s="115"/>
+      <c r="J33" s="115"/>
+      <c r="K33" s="115"/>
+      <c r="L33" s="100"/>
+      <c r="M33" s="101"/>
+      <c r="N33" s="102"/>
+      <c r="O33" s="106"/>
+      <c r="P33" s="107"/>
+      <c r="Q33" s="107"/>
+      <c r="R33" s="107"/>
+      <c r="S33" s="107"/>
+      <c r="T33" s="108"/>
       <c r="U33" s="79"/>
       <c r="V33" s="79" t="s">
         <v>91</v>
@@ -8722,29 +9106,29 @@
     </row>
     <row r="34" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A34" s="79"/>
-      <c r="B34" s="202" t="s">
+      <c r="B34" s="122" t="s">
         <v>105</v>
       </c>
-      <c r="C34" s="173"/>
-      <c r="D34" s="173"/>
-      <c r="E34" s="173"/>
-      <c r="F34" s="203"/>
-      <c r="G34" s="194" t="s">
+      <c r="C34" s="93"/>
+      <c r="D34" s="93"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="123"/>
+      <c r="G34" s="114" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="195"/>
-      <c r="I34" s="195"/>
-      <c r="J34" s="195"/>
-      <c r="K34" s="195"/>
-      <c r="L34" s="196"/>
-      <c r="M34" s="197"/>
-      <c r="N34" s="198"/>
-      <c r="O34" s="199"/>
-      <c r="P34" s="200"/>
-      <c r="Q34" s="200"/>
-      <c r="R34" s="200"/>
-      <c r="S34" s="200"/>
-      <c r="T34" s="201"/>
+      <c r="H34" s="115"/>
+      <c r="I34" s="115"/>
+      <c r="J34" s="115"/>
+      <c r="K34" s="115"/>
+      <c r="L34" s="116"/>
+      <c r="M34" s="117"/>
+      <c r="N34" s="118"/>
+      <c r="O34" s="119"/>
+      <c r="P34" s="120"/>
+      <c r="Q34" s="120"/>
+      <c r="R34" s="120"/>
+      <c r="S34" s="120"/>
+      <c r="T34" s="121"/>
       <c r="U34" s="79"/>
       <c r="V34" s="79" t="s">
         <v>94</v>
@@ -8753,29 +9137,29 @@
     </row>
     <row r="35" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A35" s="79"/>
-      <c r="B35" s="192" t="s">
+      <c r="B35" s="112" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="175"/>
-      <c r="D35" s="175"/>
-      <c r="E35" s="175"/>
-      <c r="F35" s="193"/>
-      <c r="G35" s="194" t="s">
+      <c r="C35" s="95"/>
+      <c r="D35" s="95"/>
+      <c r="E35" s="95"/>
+      <c r="F35" s="113"/>
+      <c r="G35" s="114" t="s">
         <v>108</v>
       </c>
-      <c r="H35" s="195"/>
-      <c r="I35" s="195"/>
-      <c r="J35" s="195"/>
-      <c r="K35" s="195"/>
-      <c r="L35" s="183"/>
-      <c r="M35" s="184"/>
-      <c r="N35" s="185"/>
-      <c r="O35" s="189"/>
-      <c r="P35" s="190"/>
-      <c r="Q35" s="190"/>
-      <c r="R35" s="190"/>
-      <c r="S35" s="190"/>
-      <c r="T35" s="191"/>
+      <c r="H35" s="115"/>
+      <c r="I35" s="115"/>
+      <c r="J35" s="115"/>
+      <c r="K35" s="115"/>
+      <c r="L35" s="103"/>
+      <c r="M35" s="104"/>
+      <c r="N35" s="105"/>
+      <c r="O35" s="109"/>
+      <c r="P35" s="110"/>
+      <c r="Q35" s="110"/>
+      <c r="R35" s="110"/>
+      <c r="S35" s="110"/>
+      <c r="T35" s="111"/>
       <c r="U35" s="79"/>
       <c r="V35" s="79" t="s">
         <v>97</v>
@@ -8784,54 +9168,54 @@
     </row>
     <row r="36" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A36" s="79"/>
-      <c r="B36" s="177" t="s">
+      <c r="B36" s="97" t="s">
         <v>109</v>
       </c>
-      <c r="C36" s="178"/>
-      <c r="D36" s="178"/>
-      <c r="E36" s="178"/>
-      <c r="F36" s="178"/>
-      <c r="G36" s="178"/>
-      <c r="H36" s="178"/>
-      <c r="I36" s="178"/>
-      <c r="J36" s="178"/>
-      <c r="K36" s="179"/>
-      <c r="L36" s="180"/>
-      <c r="M36" s="181"/>
-      <c r="N36" s="182"/>
-      <c r="O36" s="186"/>
-      <c r="P36" s="187"/>
-      <c r="Q36" s="187"/>
-      <c r="R36" s="187"/>
-      <c r="S36" s="187"/>
-      <c r="T36" s="188"/>
+      <c r="C36" s="98"/>
+      <c r="D36" s="98"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="98"/>
+      <c r="G36" s="98"/>
+      <c r="H36" s="98"/>
+      <c r="I36" s="98"/>
+      <c r="J36" s="98"/>
+      <c r="K36" s="99"/>
+      <c r="L36" s="100"/>
+      <c r="M36" s="101"/>
+      <c r="N36" s="102"/>
+      <c r="O36" s="106"/>
+      <c r="P36" s="107"/>
+      <c r="Q36" s="107"/>
+      <c r="R36" s="107"/>
+      <c r="S36" s="107"/>
+      <c r="T36" s="108"/>
       <c r="U36" s="79"/>
       <c r="V36" s="79"/>
       <c r="W36" s="79"/>
     </row>
     <row r="37" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A37" s="79"/>
-      <c r="B37" s="192" t="s">
+      <c r="B37" s="112" t="s">
         <v>110</v>
       </c>
-      <c r="C37" s="175"/>
-      <c r="D37" s="175"/>
-      <c r="E37" s="175"/>
-      <c r="F37" s="175"/>
-      <c r="G37" s="175"/>
-      <c r="H37" s="175"/>
-      <c r="I37" s="175"/>
-      <c r="J37" s="175"/>
-      <c r="K37" s="193"/>
-      <c r="L37" s="183"/>
-      <c r="M37" s="184"/>
-      <c r="N37" s="185"/>
-      <c r="O37" s="189"/>
-      <c r="P37" s="190"/>
-      <c r="Q37" s="190"/>
-      <c r="R37" s="190"/>
-      <c r="S37" s="190"/>
-      <c r="T37" s="191"/>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="95"/>
+      <c r="F37" s="95"/>
+      <c r="G37" s="95"/>
+      <c r="H37" s="95"/>
+      <c r="I37" s="95"/>
+      <c r="J37" s="95"/>
+      <c r="K37" s="113"/>
+      <c r="L37" s="103"/>
+      <c r="M37" s="104"/>
+      <c r="N37" s="105"/>
+      <c r="O37" s="109"/>
+      <c r="P37" s="110"/>
+      <c r="Q37" s="110"/>
+      <c r="R37" s="110"/>
+      <c r="S37" s="110"/>
+      <c r="T37" s="111"/>
       <c r="U37" s="79"/>
       <c r="V37" s="79" t="s">
         <v>128</v>
@@ -8840,54 +9224,54 @@
     </row>
     <row r="38" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A38" s="79"/>
-      <c r="B38" s="177" t="s">
+      <c r="B38" s="97" t="s">
         <v>111</v>
       </c>
-      <c r="C38" s="178"/>
-      <c r="D38" s="178"/>
-      <c r="E38" s="178"/>
-      <c r="F38" s="178"/>
-      <c r="G38" s="178"/>
-      <c r="H38" s="178"/>
-      <c r="I38" s="178"/>
-      <c r="J38" s="178"/>
-      <c r="K38" s="179"/>
-      <c r="L38" s="180"/>
-      <c r="M38" s="181"/>
-      <c r="N38" s="182"/>
-      <c r="O38" s="186"/>
-      <c r="P38" s="187"/>
-      <c r="Q38" s="187"/>
-      <c r="R38" s="187"/>
-      <c r="S38" s="187"/>
-      <c r="T38" s="188"/>
+      <c r="C38" s="98"/>
+      <c r="D38" s="98"/>
+      <c r="E38" s="98"/>
+      <c r="F38" s="98"/>
+      <c r="G38" s="98"/>
+      <c r="H38" s="98"/>
+      <c r="I38" s="98"/>
+      <c r="J38" s="98"/>
+      <c r="K38" s="99"/>
+      <c r="L38" s="100"/>
+      <c r="M38" s="101"/>
+      <c r="N38" s="102"/>
+      <c r="O38" s="106"/>
+      <c r="P38" s="107"/>
+      <c r="Q38" s="107"/>
+      <c r="R38" s="107"/>
+      <c r="S38" s="107"/>
+      <c r="T38" s="108"/>
       <c r="U38" s="79"/>
       <c r="V38" s="79"/>
       <c r="W38" s="79"/>
     </row>
     <row r="39" spans="1:23" s="81" customFormat="1" ht="12" customHeight="1">
       <c r="A39" s="79"/>
-      <c r="B39" s="192" t="s">
+      <c r="B39" s="112" t="s">
         <v>112</v>
       </c>
-      <c r="C39" s="175"/>
-      <c r="D39" s="175"/>
-      <c r="E39" s="175"/>
-      <c r="F39" s="175"/>
-      <c r="G39" s="175"/>
-      <c r="H39" s="175"/>
-      <c r="I39" s="175"/>
-      <c r="J39" s="175"/>
-      <c r="K39" s="193"/>
-      <c r="L39" s="183"/>
-      <c r="M39" s="184"/>
-      <c r="N39" s="185"/>
-      <c r="O39" s="189"/>
-      <c r="P39" s="190"/>
-      <c r="Q39" s="190"/>
-      <c r="R39" s="190"/>
-      <c r="S39" s="190"/>
-      <c r="T39" s="191"/>
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="95"/>
+      <c r="F39" s="95"/>
+      <c r="G39" s="95"/>
+      <c r="H39" s="95"/>
+      <c r="I39" s="95"/>
+      <c r="J39" s="95"/>
+      <c r="K39" s="113"/>
+      <c r="L39" s="103"/>
+      <c r="M39" s="104"/>
+      <c r="N39" s="105"/>
+      <c r="O39" s="109"/>
+      <c r="P39" s="110"/>
+      <c r="Q39" s="110"/>
+      <c r="R39" s="110"/>
+      <c r="S39" s="110"/>
+      <c r="T39" s="111"/>
       <c r="U39" s="79"/>
       <c r="V39" s="79"/>
       <c r="W39" s="79"/>
@@ -9202,20 +9586,20 @@
       <c r="F51" s="83"/>
       <c r="G51" s="83"/>
       <c r="H51" s="83"/>
-      <c r="I51" s="171" t="s">
+      <c r="I51" s="91" t="s">
         <v>122</v>
       </c>
-      <c r="J51" s="172"/>
-      <c r="K51" s="172"/>
-      <c r="L51" s="172"/>
-      <c r="M51" s="172"/>
-      <c r="N51" s="172"/>
-      <c r="O51" s="172"/>
-      <c r="P51" s="172"/>
-      <c r="Q51" s="172"/>
-      <c r="R51" s="172"/>
-      <c r="S51" s="172"/>
-      <c r="T51" s="172"/>
+      <c r="J51" s="92"/>
+      <c r="K51" s="92"/>
+      <c r="L51" s="92"/>
+      <c r="M51" s="92"/>
+      <c r="N51" s="92"/>
+      <c r="O51" s="92"/>
+      <c r="P51" s="92"/>
+      <c r="Q51" s="92"/>
+      <c r="R51" s="92"/>
+      <c r="S51" s="92"/>
+      <c r="T51" s="92"/>
       <c r="U51" s="83"/>
       <c r="V51" s="83"/>
       <c r="W51" s="83"/>
@@ -9230,19 +9614,19 @@
       <c r="G52" s="79"/>
       <c r="H52" s="79"/>
       <c r="I52" s="79"/>
-      <c r="J52" s="173" t="s">
+      <c r="J52" s="93" t="s">
         <v>123</v>
       </c>
-      <c r="K52" s="173"/>
-      <c r="L52" s="173"/>
-      <c r="M52" s="173"/>
-      <c r="N52" s="173"/>
-      <c r="O52" s="173"/>
-      <c r="P52" s="173"/>
-      <c r="Q52" s="173"/>
-      <c r="R52" s="173"/>
-      <c r="S52" s="173"/>
-      <c r="T52" s="173"/>
+      <c r="K52" s="93"/>
+      <c r="L52" s="93"/>
+      <c r="M52" s="93"/>
+      <c r="N52" s="93"/>
+      <c r="O52" s="93"/>
+      <c r="P52" s="93"/>
+      <c r="Q52" s="93"/>
+      <c r="R52" s="93"/>
+      <c r="S52" s="93"/>
+      <c r="T52" s="93"/>
       <c r="U52" s="65"/>
       <c r="V52" s="65"/>
       <c r="W52" s="65"/>
@@ -9278,54 +9662,54 @@
     </row>
     <row r="54" spans="1:23" ht="12" customHeight="1">
       <c r="A54" s="65"/>
-      <c r="B54" s="174"/>
-      <c r="C54" s="174"/>
-      <c r="D54" s="174"/>
-      <c r="E54" s="174"/>
-      <c r="F54" s="174"/>
-      <c r="G54" s="174"/>
-      <c r="H54" s="174"/>
-      <c r="I54" s="174"/>
+      <c r="B54" s="94"/>
+      <c r="C54" s="94"/>
+      <c r="D54" s="94"/>
+      <c r="E54" s="94"/>
+      <c r="F54" s="94"/>
+      <c r="G54" s="94"/>
+      <c r="H54" s="94"/>
+      <c r="I54" s="94"/>
       <c r="J54" s="65"/>
-      <c r="K54" s="169" t="s">
+      <c r="K54" s="89" t="s">
         <v>78</v>
       </c>
-      <c r="L54" s="169"/>
-      <c r="M54" s="169"/>
-      <c r="N54" s="175" t="s">
+      <c r="L54" s="89"/>
+      <c r="M54" s="89"/>
+      <c r="N54" s="95" t="s">
         <v>125</v>
       </c>
-      <c r="O54" s="175"/>
-      <c r="P54" s="175"/>
-      <c r="Q54" s="175"/>
-      <c r="R54" s="175"/>
-      <c r="S54" s="175"/>
-      <c r="T54" s="175"/>
+      <c r="O54" s="95"/>
+      <c r="P54" s="95"/>
+      <c r="Q54" s="95"/>
+      <c r="R54" s="95"/>
+      <c r="S54" s="95"/>
+      <c r="T54" s="95"/>
       <c r="U54" s="65"/>
       <c r="V54" s="65"/>
       <c r="W54" s="65"/>
     </row>
     <row r="55" spans="1:23" ht="12" customHeight="1">
       <c r="A55" s="65"/>
-      <c r="B55" s="174"/>
-      <c r="C55" s="174"/>
-      <c r="D55" s="174"/>
-      <c r="E55" s="174"/>
-      <c r="F55" s="174"/>
-      <c r="G55" s="174"/>
-      <c r="H55" s="174"/>
-      <c r="I55" s="174"/>
+      <c r="B55" s="94"/>
+      <c r="C55" s="94"/>
+      <c r="D55" s="94"/>
+      <c r="E55" s="94"/>
+      <c r="F55" s="94"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="94"/>
+      <c r="I55" s="94"/>
       <c r="J55" s="65"/>
       <c r="K55" s="65"/>
       <c r="L55" s="65"/>
       <c r="M55" s="65"/>
-      <c r="N55" s="176"/>
-      <c r="O55" s="176"/>
-      <c r="P55" s="176"/>
-      <c r="Q55" s="176"/>
-      <c r="R55" s="176"/>
-      <c r="S55" s="176"/>
-      <c r="T55" s="176"/>
+      <c r="N55" s="96"/>
+      <c r="O55" s="96"/>
+      <c r="P55" s="96"/>
+      <c r="Q55" s="96"/>
+      <c r="R55" s="96"/>
+      <c r="S55" s="96"/>
+      <c r="T55" s="96"/>
       <c r="U55" s="65"/>
       <c r="V55" s="65"/>
       <c r="W55" s="65"/>
@@ -9366,20 +9750,20 @@
       <c r="H57" s="65"/>
       <c r="I57" s="65"/>
       <c r="J57" s="65"/>
-      <c r="K57" s="169" t="s">
+      <c r="K57" s="89" t="s">
         <v>126</v>
       </c>
-      <c r="L57" s="169"/>
-      <c r="M57" s="169"/>
-      <c r="N57" s="170">
+      <c r="L57" s="89"/>
+      <c r="M57" s="89"/>
+      <c r="N57" s="90">
         <v>46236</v>
       </c>
-      <c r="O57" s="170"/>
-      <c r="P57" s="170"/>
-      <c r="Q57" s="170"/>
-      <c r="R57" s="170"/>
-      <c r="S57" s="170"/>
-      <c r="T57" s="170"/>
+      <c r="O57" s="90"/>
+      <c r="P57" s="90"/>
+      <c r="Q57" s="90"/>
+      <c r="R57" s="90"/>
+      <c r="S57" s="90"/>
+      <c r="T57" s="90"/>
       <c r="U57" s="65"/>
       <c r="V57" s="65"/>
       <c r="W57" s="65"/>

</xml_diff>